<commit_message>
(fix) Adjust Excel Chart Creation for Readability
</commit_message>
<xml_diff>
--- a/assessment/self-assessment.xlsx
+++ b/assessment/self-assessment.xlsx
@@ -521,7 +521,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -564,7 +563,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Assessment'!$C$6:$C$13</f>
+              <f>'Assessment'!$H$6:$H$13</f>
             </numRef>
           </cat>
           <val>
@@ -591,6 +590,8 @@
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
+          <max val="10"/>
+          <min val="0"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
@@ -611,7 +612,6 @@
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -630,7 +630,7 @@
     </title>
     <plotArea>
       <radarChart>
-        <radarStyle val="filled"/>
+        <radarStyle val="marker"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
@@ -654,7 +654,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Perspectives'!$C$5:$C$12</f>
+              <f>'Perspectives'!$M$5:$M$12</f>
             </numRef>
           </cat>
           <val>
@@ -686,7 +686,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Perspectives'!$C$5:$C$12</f>
+              <f>'Perspectives'!$M$5:$M$12</f>
             </numRef>
           </cat>
           <val>
@@ -718,7 +718,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Perspectives'!$C$5:$C$12</f>
+              <f>'Perspectives'!$M$5:$M$12</f>
             </numRef>
           </cat>
           <val>
@@ -750,7 +750,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Perspectives'!$C$5:$C$12</f>
+              <f>'Perspectives'!$M$5:$M$12</f>
             </numRef>
           </cat>
           <val>
@@ -782,7 +782,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Perspectives'!$C$5:$C$12</f>
+              <f>'Perspectives'!$M$5:$M$12</f>
             </numRef>
           </cat>
           <val>
@@ -814,7 +814,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Perspectives'!$C$5:$C$12</f>
+              <f>'Perspectives'!$M$5:$M$12</f>
             </numRef>
           </cat>
           <val>
@@ -846,7 +846,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Perspectives'!$C$5:$C$12</f>
+              <f>'Perspectives'!$M$5:$M$12</f>
             </numRef>
           </cat>
           <val>
@@ -878,7 +878,7 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Perspectives'!$C$5:$C$12</f>
+              <f>'Perspectives'!$M$5:$M$12</f>
             </numRef>
           </cat>
           <val>
@@ -905,6 +905,8 @@
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
+          <max val="10"/>
+          <min val="0"/>
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
@@ -926,12 +928,12 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>7</col>
+      <col>8</col>
       <colOff>0</colOff>
-      <row>5</row>
+      <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6480000" cy="5760000"/>
+    <ext cx="7920000" cy="7200000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -953,12 +955,12 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>13</col>
+      <col>14</col>
       <colOff>0</colOff>
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7200000" cy="6480000"/>
+    <ext cx="8640000" cy="7920000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -1285,7 +1287,7 @@
     <row r="3" ht="22" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Building Automation Muscle Without a Dev Team  ·  MSP/ITSP Framework</t>
+          <t>A Team Capability Framework  ·  8 Dimensions of Automation Readiness</t>
         </is>
       </c>
     </row>
@@ -1299,14 +1301,14 @@
     <row r="6" ht="15" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>This workbook supports the Archetypes of Automation framework — a team capability assessment tool for MSP/ITSP leaders. It is designed to be completed by a key team member or person in a position of authority evaluating their team's collective strengths and gaps.</t>
+          <t>This workbook supports the Archetypes of Automation framework — a team capability assessment tool for any organisation building automation capabilities. It is designed to be completed by a team leader or person in a position of authority evaluating their team's collective strengths and gaps.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>The biggest barrier to automation in small MSP teams is not technical skill — it is process thinking, team composition, and role awareness. This tool helps you see where your team stands across 8 automation capability dimensions.</t>
+          <t>The biggest barrier to automation is not technical skill — it is process thinking, team composition, and role awareness. This tool helps you see where your team stands across 8 automation capability dimensions.</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:F16"/>
+  <dimension ref="B1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1595,6 +1597,7 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="28" customWidth="1" min="6" max="6"/>
     <col width="3" customWidth="1" min="7" max="7"/>
+    <col hidden="1" width="18" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1665,6 +1668,11 @@
         <f>IF(E6&lt;=2,"0-2: No one on the team fills this role; capability absent",IF(E6&lt;=4,"3-4: Emerging - someone shows instinct but no structured practice",IF(E6&lt;=6,"5-6: Functional - team has some coverage but with notable gaps",IF(E6&lt;=8,"7-8: Strong - reliable team capability; people know who to go to","9-10: Exceptional - a clear team strength; you set the standard"))))</f>
         <v/>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>1. Process</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="36" customHeight="1">
       <c r="B7" s="10" t="n">
@@ -1687,6 +1695,11 @@
         <f>IF(E7&lt;=2,"0-2: No one on the team fills this role; capability absent",IF(E7&lt;=4,"3-4: Emerging - someone shows instinct but no structured practice",IF(E7&lt;=6,"5-6: Functional - team has some coverage but with notable gaps",IF(E7&lt;=8,"7-8: Strong - reliable team capability; people know who to go to","9-10: Exceptional - a clear team strength; you set the standard"))))</f>
         <v/>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2. Problem Def.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="36" customHeight="1">
       <c r="B8" s="10" t="n">
@@ -1709,6 +1722,11 @@
         <f>IF(E8&lt;=2,"0-2: No one on the team fills this role; capability absent",IF(E8&lt;=4,"3-4: Emerging - someone shows instinct but no structured practice",IF(E8&lt;=6,"5-6: Functional - team has some coverage but with notable gaps",IF(E8&lt;=8,"7-8: Strong - reliable team capability; people know who to go to","9-10: Exceptional - a clear team strength; you set the standard"))))</f>
         <v/>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>3. Design &amp; Logic</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="36" customHeight="1">
       <c r="B9" s="10" t="n">
@@ -1731,6 +1749,11 @@
         <f>IF(E9&lt;=2,"0-2: No one on the team fills this role; capability absent",IF(E9&lt;=4,"3-4: Emerging - someone shows instinct but no structured practice",IF(E9&lt;=6,"5-6: Functional - team has some coverage but with notable gaps",IF(E9&lt;=8,"7-8: Strong - reliable team capability; people know who to go to","9-10: Exceptional - a clear team strength; you set the standard"))))</f>
         <v/>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>4. Communication</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="36" customHeight="1">
       <c r="B10" s="10" t="n">
@@ -1753,6 +1776,11 @@
         <f>IF(E10&lt;=2,"0-2: No one on the team fills this role; capability absent",IF(E10&lt;=4,"3-4: Emerging - someone shows instinct but no structured practice",IF(E10&lt;=6,"5-6: Functional - team has some coverage but with notable gaps",IF(E10&lt;=8,"7-8: Strong - reliable team capability; people know who to go to","9-10: Exceptional - a clear team strength; you set the standard"))))</f>
         <v/>
       </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>5. Building</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="36" customHeight="1">
       <c r="B11" s="10" t="n">
@@ -1775,6 +1803,11 @@
         <f>IF(E11&lt;=2,"0-2: No one on the team fills this role; capability absent",IF(E11&lt;=4,"3-4: Emerging - someone shows instinct but no structured practice",IF(E11&lt;=6,"5-6: Functional - team has some coverage but with notable gaps",IF(E11&lt;=8,"7-8: Strong - reliable team capability; people know who to go to","9-10: Exceptional - a clear team strength; you set the standard"))))</f>
         <v/>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>6. Quality</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="36" customHeight="1">
       <c r="B12" s="10" t="n">
@@ -1797,6 +1830,11 @@
         <f>IF(E12&lt;=2,"0-2: No one on the team fills this role; capability absent",IF(E12&lt;=4,"3-4: Emerging - someone shows instinct but no structured practice",IF(E12&lt;=6,"5-6: Functional - team has some coverage but with notable gaps",IF(E12&lt;=8,"7-8: Strong - reliable team capability; people know who to go to","9-10: Exceptional - a clear team strength; you set the standard"))))</f>
         <v/>
       </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>7. People &amp; Org.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="36" customHeight="1">
       <c r="B13" s="10" t="n">
@@ -1818,6 +1856,11 @@
       <c r="F13" s="17">
         <f>IF(E13&lt;=2,"0-2: No one on the team fills this role; capability absent",IF(E13&lt;=4,"3-4: Emerging - someone shows instinct but no structured practice",IF(E13&lt;=6,"5-6: Functional - team has some coverage but with notable gaps",IF(E13&lt;=8,"7-8: Strong - reliable team capability; people know who to go to","9-10: Exceptional - a clear team strength; you set the standard"))))</f>
         <v/>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>8. Strategy</t>
+        </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
@@ -1881,7 +1924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:L23"/>
+  <dimension ref="B1:M23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1896,7 +1939,7 @@
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="3" customWidth="1" min="13" max="13"/>
+    <col hidden="1" width="18" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -2049,6 +2092,11 @@
         <f>AVERAGE(D5:K5)</f>
         <v/>
       </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>1. Process</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="B6" s="10" t="n">
@@ -2087,6 +2135,11 @@
         <f>AVERAGE(D6:K6)</f>
         <v/>
       </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2. Problem Def.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="10" t="n">
@@ -2125,6 +2178,11 @@
         <f>AVERAGE(D7:K7)</f>
         <v/>
       </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>3. Design &amp; Logic</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="B8" s="10" t="n">
@@ -2163,6 +2221,11 @@
         <f>AVERAGE(D8:K8)</f>
         <v/>
       </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>4. Communication</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="B9" s="10" t="n">
@@ -2201,6 +2264,11 @@
         <f>AVERAGE(D9:K9)</f>
         <v/>
       </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>5. Building</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="B10" s="10" t="n">
@@ -2239,6 +2307,11 @@
         <f>AVERAGE(D10:K10)</f>
         <v/>
       </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>6. Quality</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="B11" s="10" t="n">
@@ -2277,6 +2350,11 @@
         <f>AVERAGE(D11:K11)</f>
         <v/>
       </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>7. People &amp; Org.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="B12" s="10" t="n">
@@ -2314,6 +2392,11 @@
       <c r="L12" s="29">
         <f>AVERAGE(D12:K12)</f>
         <v/>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>8. Strategy</t>
+        </is>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">

</xml_diff>